<commit_message>
Merge parcel into approved design plots, refactor case views, and sync requirements.
Consolidate allocation on approved design plots with data migrations, split cases views into modules, improve application import, and update specs and tests.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/application_import_appendix3_v1.0.1_SAMPLE.xlsx
+++ b/application_import_appendix3_v1.0.1_SAMPLE.xlsx
@@ -71,9 +71,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -533,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18.8" customWidth="1" min="1" max="1"/>
@@ -559,33 +560,633 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>document_code</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>document_status</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>document_comments</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Από κατάλογο συστήματος</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>ΝΑΙ | ΟΧΙ | ΔΕΝ ΑΠΑΙΤΕΙΤΑΙ</t>
         </is>
       </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="n"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="n"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="n"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="n"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="n"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="n"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="n"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="n"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="n"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="n"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="n"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="n"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="n"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="n"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="n"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="n"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="n"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="n"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="n"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="n"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="n"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="n"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="n"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="n"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="n"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="n"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="n"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="n"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="n"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="n"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="n"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="n"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="n"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="n"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="n"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="n"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="n"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="n"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="n"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="n"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="n"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="n"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="n"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="n"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="n"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="n"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="n"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="n"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="n"/>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="n"/>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="n"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="n"/>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="n"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="n"/>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="n"/>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="n"/>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="n"/>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="n"/>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="n"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="2" t="n"/>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="n"/>
+    </row>
+    <row r="191">
+      <c r="A191" s="2" t="n"/>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="n"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="n"/>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="n"/>
+    </row>
+    <row r="195">
+      <c r="A195" s="2" t="n"/>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="n"/>
+    </row>
+    <row r="197">
+      <c r="A197" s="2" t="n"/>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="n"/>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="n"/>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="n"/>
+    </row>
+    <row r="201">
+      <c r="A201" s="2" t="n"/>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="n"/>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -668,7 +1269,7 @@
           <t>Κωδικός Κοινότητας / Δ.Δ. (Παράρτημα 1)</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>001</t>
         </is>
@@ -702,7 +1303,7 @@
           <t>Αρ. πρωτοκόλλησης (επίσημη χρήση)</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>ΠΡΩΤ-2026-0042</t>
         </is>
@@ -753,166 +1354,166 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Ημερομηνία υποβολής αίτησης</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Ηλεκτρονική διεύθυνση αιτητή</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Τύπος οικογένειας</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Τύπος οικογένειας — Άλλο (κείμενο)</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Αριθμός τέκνων (δήλωση)</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Έγγαμος</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Σύμφωνο συμβίωσης</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Μονογονεϊκή οικογένεια</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Χήρος/α</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Διαζευγμένος/η</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>Σχόλια λειτουργού</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>submitted_on</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>applicant_email</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>family_type</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>family_type_other</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>declared_children_count</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>family_married</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>family_civil_union</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>family_single_parent</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>family_widow</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="J2" s="4" t="inlineStr">
         <is>
           <t>family_divorced</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="K2" s="4" t="inlineStr">
         <is>
           <t>comments</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>YYYY-MM-DD · 10.1</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>10.1 · επίσημη επικοινωνία</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>with_children | couple_no_children | single_parent | other</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>Αν family_type=other</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>Ακέραιος</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>Ναι | Όχι</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>Ναι | Όχι</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>Ναι | Όχι</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="I3" s="5" t="inlineStr">
         <is>
           <t>Ναι | Όχι</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="J3" s="5" t="inlineStr">
         <is>
           <t>Ναι | Όχι</t>
         </is>
@@ -1013,301 +1614,301 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Όνομα αιτητή/αιτήτριας</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Επίθετο</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Αρ. Δελτίου Ταυτότητας</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Αρ. Κοινωνικών Ασφαλίσεων</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Αρ. Προσφυγικής Ταυτότητας</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Κύπριος Πολίτης</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Επαναπατρισθείς/είσα Κύπριος/α</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Ημερομηνία γέννησης</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Τόπος γέννησης</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Χώρα γέννησης</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>Τόπος γέννησης γονέων</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>Χώρα γέννησης γονέων</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>Τηλέφωνο κινητό</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>Τηλέφωνο σταθερό</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>Διεύθυνση αλληλογραφίας — Οδός</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>Διεύθυνση αλληλογραφίας — Αριθμός</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>Διεύθυνση αλληλογραφίας — Διαμέρισμα</t>
         </is>
       </c>
-      <c r="R1" s="2" t="inlineStr">
+      <c r="R1" s="3" t="inlineStr">
         <is>
           <t>Διεύθυνση αλληλογραφίας — Κοινότητα/Δ.Δ.</t>
         </is>
       </c>
-      <c r="S1" s="2" t="inlineStr">
+      <c r="S1" s="3" t="inlineStr">
         <is>
           <t>Διεύθυνση αλληλογραφίας — Ταχ. κωδ.</t>
         </is>
       </c>
-      <c r="T1" s="2" t="inlineStr">
+      <c r="T1" s="3" t="inlineStr">
         <is>
           <t>Διεύθυνση αλληλογραφίας — Επαρχία</t>
         </is>
       </c>
-      <c r="U1" s="2" t="inlineStr">
+      <c r="U1" s="3" t="inlineStr">
         <is>
           <t>Επαγγελματική κατάσταση — Αυτοτελώς εργαζόμενος</t>
         </is>
       </c>
-      <c r="V1" s="2" t="inlineStr">
+      <c r="V1" s="3" t="inlineStr">
         <is>
           <t>Επαγγελματική κατάσταση — Μισθωτός</t>
         </is>
       </c>
-      <c r="W1" s="2" t="inlineStr">
+      <c r="W1" s="3" t="inlineStr">
         <is>
           <t>Επαγγελματική κατάσταση — Άνεργος</t>
         </is>
       </c>
-      <c r="X1" s="2" t="inlineStr">
+      <c r="X1" s="3" t="inlineStr">
         <is>
           <t>Επαγγελματική κατάσταση — Άτομο με αναπηρία</t>
         </is>
       </c>
-      <c r="Y1" s="2" t="inlineStr">
+      <c r="Y1" s="3" t="inlineStr">
         <is>
           <t>Εργοδότης (πληροφορίες)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>p1_first_name</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>p1_last_name</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>p1_identity_number</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>p1_social_insurance_number</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>p1_refugee_id</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>p1_citizenship_cypriot</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>p1_citizenship_repatriated</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>p1_date_of_birth</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>p1_birth_place</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="J2" s="4" t="inlineStr">
         <is>
           <t>p1_birth_country</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="K2" s="4" t="inlineStr">
         <is>
           <t>p1_parents_birth_place</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="L2" s="4" t="inlineStr">
         <is>
           <t>p1_parents_birth_country</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="M2" s="4" t="inlineStr">
         <is>
           <t>p1_mobile_phone</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="N2" s="4" t="inlineStr">
         <is>
           <t>p1_landline_phone</t>
         </is>
       </c>
-      <c r="O2" s="3" t="inlineStr">
+      <c r="O2" s="4" t="inlineStr">
         <is>
           <t>p1_mailing_street</t>
         </is>
       </c>
-      <c r="P2" s="3" t="inlineStr">
+      <c r="P2" s="4" t="inlineStr">
         <is>
           <t>p1_mailing_number</t>
         </is>
       </c>
-      <c r="Q2" s="3" t="inlineStr">
+      <c r="Q2" s="4" t="inlineStr">
         <is>
           <t>p1_mailing_apartment</t>
         </is>
       </c>
-      <c r="R2" s="3" t="inlineStr">
+      <c r="R2" s="4" t="inlineStr">
         <is>
           <t>p1_mailing_community</t>
         </is>
       </c>
-      <c r="S2" s="3" t="inlineStr">
+      <c r="S2" s="4" t="inlineStr">
         <is>
           <t>p1_mailing_postal_code</t>
         </is>
       </c>
-      <c r="T2" s="3" t="inlineStr">
+      <c r="T2" s="4" t="inlineStr">
         <is>
           <t>p1_mailing_district</t>
         </is>
       </c>
-      <c r="U2" s="3" t="inlineStr">
+      <c r="U2" s="4" t="inlineStr">
         <is>
           <t>p1_employment_self_employed</t>
         </is>
       </c>
-      <c r="V2" s="3" t="inlineStr">
+      <c r="V2" s="4" t="inlineStr">
         <is>
           <t>p1_employment_employee</t>
         </is>
       </c>
-      <c r="W2" s="3" t="inlineStr">
+      <c r="W2" s="4" t="inlineStr">
         <is>
           <t>p1_employment_unemployed</t>
         </is>
       </c>
-      <c r="X2" s="3" t="inlineStr">
+      <c r="X2" s="4" t="inlineStr">
         <is>
           <t>p1_employment_disability</t>
         </is>
       </c>
-      <c r="Y2" s="3" t="inlineStr">
+      <c r="Y2" s="4" t="inlineStr">
         <is>
           <t>p1_employer_info</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>Υποχρεωτικό</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>Όπου εφαρμόζεται</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>Ναι | Όχι</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>Ναι | Όχι</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>YYYY-MM-DD</t>
         </is>
       </c>
-      <c r="U3" s="4" t="inlineStr">
+      <c r="U3" s="5" t="inlineStr">
         <is>
           <t>Ναι | Όχι</t>
         </is>
       </c>
-      <c r="V3" s="4" t="inlineStr">
+      <c r="V3" s="5" t="inlineStr">
         <is>
           <t>Ναι | Όχι</t>
         </is>
       </c>
-      <c r="W3" s="4" t="inlineStr">
+      <c r="W3" s="5" t="inlineStr">
         <is>
           <t>Ναι | Όχι</t>
         </is>
       </c>
-      <c r="X3" s="4" t="inlineStr">
+      <c r="X3" s="5" t="inlineStr">
         <is>
           <t>Ναι | Όχι</t>
         </is>
@@ -1324,17 +1925,17 @@
           <t>Παπαδόπουλος</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>K123456</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>1234567890</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>Ναι</t>
@@ -1370,12 +1971,12 @@
           <t>Κύπρος</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>99123456</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>22456789</t>
         </is>
@@ -1396,7 +1997,7 @@
           <t>Αγία Βαρβάρα</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="S4" s="2" t="inlineStr">
         <is>
           <t>2700</t>
         </is>
@@ -1471,271 +2072,271 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Όνομα συζύγου/συμβίου</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Επίθετο</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Αρ. Δελτίου Ταυτότητας</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Αρ. Κοινωνικών Ασφαλίσεων</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Αρ. Προσφυγικής Ταυτότητας</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Alien Registration Certificate</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Κύπριος Πολίτης</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Πολίτης κράτους μέλους ΕΕ</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Άλλη υπηκοότητα (κείμενο)</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Επαναπατρισθείς/είσα Κύπριος/α</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>Ημερομηνία γέννησης</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>Τόπος γέννησης</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>Χώρα γέννησης</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>Τόπος γέννησης γονέων</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>Χώρα γέννησης γονέων</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>Τηλέφωνο κινητό</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>Τηλέφωνο σταθερό</t>
         </is>
       </c>
-      <c r="R1" s="2" t="inlineStr">
+      <c r="R1" s="3" t="inlineStr">
         <is>
           <t>Επαγγελματική κατάσταση — Αυτοτελώς εργαζόμενος</t>
         </is>
       </c>
-      <c r="S1" s="2" t="inlineStr">
+      <c r="S1" s="3" t="inlineStr">
         <is>
           <t>Επαγγελματική κατάσταση — Μισθωτός</t>
         </is>
       </c>
-      <c r="T1" s="2" t="inlineStr">
+      <c r="T1" s="3" t="inlineStr">
         <is>
           <t>Επαγγελματική κατάσταση — Άνεργος</t>
         </is>
       </c>
-      <c r="U1" s="2" t="inlineStr">
+      <c r="U1" s="3" t="inlineStr">
         <is>
           <t>Επαγγελματική κατάσταση — Άτομο με αναπηρία</t>
         </is>
       </c>
-      <c r="V1" s="2" t="inlineStr">
+      <c r="V1" s="3" t="inlineStr">
         <is>
           <t>Εργοδότης (πληροφορίες)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>p2_first_name</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>p2_last_name</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>p2_identity_number</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>p2_social_insurance_number</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>p2_refugee_id</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>p2_alien_registration</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>p2_citizenship_cypriot</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>p2_citizenship_eu</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>p2_citizenship_other</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="J2" s="4" t="inlineStr">
         <is>
           <t>p2_citizenship_repatriated</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="K2" s="4" t="inlineStr">
         <is>
           <t>p2_date_of_birth</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="L2" s="4" t="inlineStr">
         <is>
           <t>p2_birth_place</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="M2" s="4" t="inlineStr">
         <is>
           <t>p2_birth_country</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="N2" s="4" t="inlineStr">
         <is>
           <t>p2_parents_birth_place</t>
         </is>
       </c>
-      <c r="O2" s="3" t="inlineStr">
+      <c r="O2" s="4" t="inlineStr">
         <is>
           <t>p2_parents_birth_country</t>
         </is>
       </c>
-      <c r="P2" s="3" t="inlineStr">
+      <c r="P2" s="4" t="inlineStr">
         <is>
           <t>p2_mobile_phone</t>
         </is>
       </c>
-      <c r="Q2" s="3" t="inlineStr">
+      <c r="Q2" s="4" t="inlineStr">
         <is>
           <t>p2_landline_phone</t>
         </is>
       </c>
-      <c r="R2" s="3" t="inlineStr">
+      <c r="R2" s="4" t="inlineStr">
         <is>
           <t>p2_employment_self_employed</t>
         </is>
       </c>
-      <c r="S2" s="3" t="inlineStr">
+      <c r="S2" s="4" t="inlineStr">
         <is>
           <t>p2_employment_employee</t>
         </is>
       </c>
-      <c r="T2" s="3" t="inlineStr">
+      <c r="T2" s="4" t="inlineStr">
         <is>
           <t>p2_employment_unemployed</t>
         </is>
       </c>
-      <c r="U2" s="3" t="inlineStr">
+      <c r="U2" s="4" t="inlineStr">
         <is>
           <t>p2_employment_disability</t>
         </is>
       </c>
-      <c r="V2" s="3" t="inlineStr">
+      <c r="V2" s="4" t="inlineStr">
         <is>
           <t>p2_employer_info</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>Όπου εφαρμόζεται</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>Ναι | Όχι</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>Ναι | Όχι</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="J3" s="5" t="inlineStr">
         <is>
           <t>Ναι | Όχι</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="K3" s="5" t="inlineStr">
         <is>
           <t>YYYY-MM-DD</t>
         </is>
       </c>
-      <c r="R3" s="4" t="inlineStr">
+      <c r="R3" s="5" t="inlineStr">
         <is>
           <t>Ναι | Όχι</t>
         </is>
       </c>
-      <c r="S3" s="4" t="inlineStr">
+      <c r="S3" s="5" t="inlineStr">
         <is>
           <t>Ναι | Όχι</t>
         </is>
       </c>
-      <c r="T3" s="4" t="inlineStr">
+      <c r="T3" s="5" t="inlineStr">
         <is>
           <t>Ναι | Όχι</t>
         </is>
       </c>
-      <c r="U3" s="4" t="inlineStr">
+      <c r="U3" s="5" t="inlineStr">
         <is>
           <t>Ναι | Όχι</t>
         </is>
@@ -1752,18 +2353,18 @@
           <t>Παπαδόπουλου</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>K654321</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>0987654321</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>Ναι</t>
@@ -1805,12 +2406,12 @@
           <t>Κύπρος</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="P4" s="2" t="inlineStr">
         <is>
           <t>99765432</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr"/>
+      <c r="Q4" s="2" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
           <t>Όχι</t>
@@ -1871,231 +2472,231 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Κατηγορία διαμονής (10.4.3)</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Τόπος διαμονής Π1 — Οδός</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Τόπος διαμονής Π1 — Αριθμός</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Τόπος διαμονής Π1 — Διαμέρισμα</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Τόπος διαμονής Π1 — Κοινότητα/Δ.Δ.</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Τόπος διαμονής Π1 — Ταχ. κωδ.</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Τόπος διαμονής Π1 — Έναρξη διαμονής</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Π1 — Περιγραφή περιόδων διαμονής / διακοπών</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Π1 — Καταγωγή από κοινότητα (ποιος γονέας)</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Π1 — Διεύθυνση στην κοινότητα (παλαιά διαμονή)</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>Π1 — Περίοδος μόνιμης κατοίκησης στην κοινότητα</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>Π1 — Τριετής διαμονή (κατ. Γ α)</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>Π1 — Δεκαετής παραμονή εξωτερικού (κατ. Γ β)</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>Γειτονική κοινότητα (κατ. Δ)</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>Τόπος διαμονής Π2 — Κοινότητα/Δ.Δ.</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>Τόπος διαμονής Π2 — Διεύθυνση (πλήρης)</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>Τόπος διαμονής Π2 — Έναρξη διαμονής</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>residence_category</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>p1_residence_street</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>p1_residence_number</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>p1_residence_apartment</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>p1_residence_community</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>p1_residence_postal_code</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>p1_residence_start</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>p1_residence_period_notes</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>p1_residence_origin_parent</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="J2" s="4" t="inlineStr">
         <is>
           <t>p1_residence_past_community_address</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="K2" s="4" t="inlineStr">
         <is>
           <t>p1_residence_past_period</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="L2" s="4" t="inlineStr">
         <is>
           <t>p1_residence_three_year_period</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="M2" s="4" t="inlineStr">
         <is>
           <t>p1_residence_ten_year_abroad</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="N2" s="4" t="inlineStr">
         <is>
           <t>neighbor_community_name</t>
         </is>
       </c>
-      <c r="O2" s="3" t="inlineStr">
+      <c r="O2" s="4" t="inlineStr">
         <is>
           <t>p2_residence_community</t>
         </is>
       </c>
-      <c r="P2" s="3" t="inlineStr">
+      <c r="P2" s="4" t="inlineStr">
         <is>
           <t>p2_residence_address</t>
         </is>
       </c>
-      <c r="Q2" s="3" t="inlineStr">
+      <c r="Q2" s="4" t="inlineStr">
         <is>
           <t>p2_residence_start</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>A | B | C | D (Αυτόχθονας/Εκτοπισθείς | Απόδημος εσωτερικού | Επαναπατρισθείς/απόδημος εξωτερικού | Γειτονική κοινότητα)</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>10.3.4</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>YYYY-MM-DD</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>Ενότητα 2 Παράρτημα 3</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="I3" s="5" t="inlineStr">
         <is>
           <t>Κατηγορία Β</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="J3" s="5" t="inlineStr">
         <is>
           <t>Κατηγορία Β</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="K3" s="5" t="inlineStr">
         <is>
           <t>από-μέχρι</t>
         </is>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="L3" s="5" t="inlineStr">
         <is>
           <t>από-μέχρι</t>
         </is>
       </c>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="M3" s="5" t="inlineStr">
         <is>
           <t>από-μέχρι</t>
         </is>
       </c>
-      <c r="N3" s="4" t="inlineStr">
+      <c r="N3" s="5" t="inlineStr">
         <is>
           <t>Από κατάλογο 15 χλμ.</t>
         </is>
       </c>
-      <c r="Q3" s="4" t="inlineStr">
+      <c r="Q3" s="5" t="inlineStr">
         <is>
           <t>YYYY-MM-DD</t>
         </is>
@@ -2123,7 +2724,7 @@
           <t>Αγία Βαρβάρα</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>2700</t>
         </is>
@@ -2167,7 +2768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2217,54 +2818,54 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>child_seq</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>child_first_name</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>child_last_name</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>child_date_of_birth</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>child_identity_number</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>child_status</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>child_is_recognized_dependent</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>YYYY-MM-DD</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>minor | student | national_guard | adult_disability</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>Ναι | Όχι</t>
         </is>
@@ -2291,7 +2892,7 @@
           <t>2014-11-05</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>minor</t>
@@ -2302,6 +2903,603 @@
           <t>Ναι</t>
         </is>
       </c>
+    </row>
+    <row r="5">
+      <c r="E5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="E6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="E7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="E8" s="2" t="n"/>
+    </row>
+    <row r="9">
+      <c r="E9" s="2" t="n"/>
+    </row>
+    <row r="10">
+      <c r="E10" s="2" t="n"/>
+    </row>
+    <row r="11">
+      <c r="E11" s="2" t="n"/>
+    </row>
+    <row r="12">
+      <c r="E12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="E13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="E14" s="2" t="n"/>
+    </row>
+    <row r="15">
+      <c r="E15" s="2" t="n"/>
+    </row>
+    <row r="16">
+      <c r="E16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="E17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="E18" s="2" t="n"/>
+    </row>
+    <row r="19">
+      <c r="E19" s="2" t="n"/>
+    </row>
+    <row r="20">
+      <c r="E20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="E21" s="2" t="n"/>
+    </row>
+    <row r="22">
+      <c r="E22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="E23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="E24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="E25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="E26" s="2" t="n"/>
+    </row>
+    <row r="27">
+      <c r="E27" s="2" t="n"/>
+    </row>
+    <row r="28">
+      <c r="E28" s="2" t="n"/>
+    </row>
+    <row r="29">
+      <c r="E29" s="2" t="n"/>
+    </row>
+    <row r="30">
+      <c r="E30" s="2" t="n"/>
+    </row>
+    <row r="31">
+      <c r="E31" s="2" t="n"/>
+    </row>
+    <row r="32">
+      <c r="E32" s="2" t="n"/>
+    </row>
+    <row r="33">
+      <c r="E33" s="2" t="n"/>
+    </row>
+    <row r="34">
+      <c r="E34" s="2" t="n"/>
+    </row>
+    <row r="35">
+      <c r="E35" s="2" t="n"/>
+    </row>
+    <row r="36">
+      <c r="E36" s="2" t="n"/>
+    </row>
+    <row r="37">
+      <c r="E37" s="2" t="n"/>
+    </row>
+    <row r="38">
+      <c r="E38" s="2" t="n"/>
+    </row>
+    <row r="39">
+      <c r="E39" s="2" t="n"/>
+    </row>
+    <row r="40">
+      <c r="E40" s="2" t="n"/>
+    </row>
+    <row r="41">
+      <c r="E41" s="2" t="n"/>
+    </row>
+    <row r="42">
+      <c r="E42" s="2" t="n"/>
+    </row>
+    <row r="43">
+      <c r="E43" s="2" t="n"/>
+    </row>
+    <row r="44">
+      <c r="E44" s="2" t="n"/>
+    </row>
+    <row r="45">
+      <c r="E45" s="2" t="n"/>
+    </row>
+    <row r="46">
+      <c r="E46" s="2" t="n"/>
+    </row>
+    <row r="47">
+      <c r="E47" s="2" t="n"/>
+    </row>
+    <row r="48">
+      <c r="E48" s="2" t="n"/>
+    </row>
+    <row r="49">
+      <c r="E49" s="2" t="n"/>
+    </row>
+    <row r="50">
+      <c r="E50" s="2" t="n"/>
+    </row>
+    <row r="51">
+      <c r="E51" s="2" t="n"/>
+    </row>
+    <row r="52">
+      <c r="E52" s="2" t="n"/>
+    </row>
+    <row r="53">
+      <c r="E53" s="2" t="n"/>
+    </row>
+    <row r="54">
+      <c r="E54" s="2" t="n"/>
+    </row>
+    <row r="55">
+      <c r="E55" s="2" t="n"/>
+    </row>
+    <row r="56">
+      <c r="E56" s="2" t="n"/>
+    </row>
+    <row r="57">
+      <c r="E57" s="2" t="n"/>
+    </row>
+    <row r="58">
+      <c r="E58" s="2" t="n"/>
+    </row>
+    <row r="59">
+      <c r="E59" s="2" t="n"/>
+    </row>
+    <row r="60">
+      <c r="E60" s="2" t="n"/>
+    </row>
+    <row r="61">
+      <c r="E61" s="2" t="n"/>
+    </row>
+    <row r="62">
+      <c r="E62" s="2" t="n"/>
+    </row>
+    <row r="63">
+      <c r="E63" s="2" t="n"/>
+    </row>
+    <row r="64">
+      <c r="E64" s="2" t="n"/>
+    </row>
+    <row r="65">
+      <c r="E65" s="2" t="n"/>
+    </row>
+    <row r="66">
+      <c r="E66" s="2" t="n"/>
+    </row>
+    <row r="67">
+      <c r="E67" s="2" t="n"/>
+    </row>
+    <row r="68">
+      <c r="E68" s="2" t="n"/>
+    </row>
+    <row r="69">
+      <c r="E69" s="2" t="n"/>
+    </row>
+    <row r="70">
+      <c r="E70" s="2" t="n"/>
+    </row>
+    <row r="71">
+      <c r="E71" s="2" t="n"/>
+    </row>
+    <row r="72">
+      <c r="E72" s="2" t="n"/>
+    </row>
+    <row r="73">
+      <c r="E73" s="2" t="n"/>
+    </row>
+    <row r="74">
+      <c r="E74" s="2" t="n"/>
+    </row>
+    <row r="75">
+      <c r="E75" s="2" t="n"/>
+    </row>
+    <row r="76">
+      <c r="E76" s="2" t="n"/>
+    </row>
+    <row r="77">
+      <c r="E77" s="2" t="n"/>
+    </row>
+    <row r="78">
+      <c r="E78" s="2" t="n"/>
+    </row>
+    <row r="79">
+      <c r="E79" s="2" t="n"/>
+    </row>
+    <row r="80">
+      <c r="E80" s="2" t="n"/>
+    </row>
+    <row r="81">
+      <c r="E81" s="2" t="n"/>
+    </row>
+    <row r="82">
+      <c r="E82" s="2" t="n"/>
+    </row>
+    <row r="83">
+      <c r="E83" s="2" t="n"/>
+    </row>
+    <row r="84">
+      <c r="E84" s="2" t="n"/>
+    </row>
+    <row r="85">
+      <c r="E85" s="2" t="n"/>
+    </row>
+    <row r="86">
+      <c r="E86" s="2" t="n"/>
+    </row>
+    <row r="87">
+      <c r="E87" s="2" t="n"/>
+    </row>
+    <row r="88">
+      <c r="E88" s="2" t="n"/>
+    </row>
+    <row r="89">
+      <c r="E89" s="2" t="n"/>
+    </row>
+    <row r="90">
+      <c r="E90" s="2" t="n"/>
+    </row>
+    <row r="91">
+      <c r="E91" s="2" t="n"/>
+    </row>
+    <row r="92">
+      <c r="E92" s="2" t="n"/>
+    </row>
+    <row r="93">
+      <c r="E93" s="2" t="n"/>
+    </row>
+    <row r="94">
+      <c r="E94" s="2" t="n"/>
+    </row>
+    <row r="95">
+      <c r="E95" s="2" t="n"/>
+    </row>
+    <row r="96">
+      <c r="E96" s="2" t="n"/>
+    </row>
+    <row r="97">
+      <c r="E97" s="2" t="n"/>
+    </row>
+    <row r="98">
+      <c r="E98" s="2" t="n"/>
+    </row>
+    <row r="99">
+      <c r="E99" s="2" t="n"/>
+    </row>
+    <row r="100">
+      <c r="E100" s="2" t="n"/>
+    </row>
+    <row r="101">
+      <c r="E101" s="2" t="n"/>
+    </row>
+    <row r="102">
+      <c r="E102" s="2" t="n"/>
+    </row>
+    <row r="103">
+      <c r="E103" s="2" t="n"/>
+    </row>
+    <row r="104">
+      <c r="E104" s="2" t="n"/>
+    </row>
+    <row r="105">
+      <c r="E105" s="2" t="n"/>
+    </row>
+    <row r="106">
+      <c r="E106" s="2" t="n"/>
+    </row>
+    <row r="107">
+      <c r="E107" s="2" t="n"/>
+    </row>
+    <row r="108">
+      <c r="E108" s="2" t="n"/>
+    </row>
+    <row r="109">
+      <c r="E109" s="2" t="n"/>
+    </row>
+    <row r="110">
+      <c r="E110" s="2" t="n"/>
+    </row>
+    <row r="111">
+      <c r="E111" s="2" t="n"/>
+    </row>
+    <row r="112">
+      <c r="E112" s="2" t="n"/>
+    </row>
+    <row r="113">
+      <c r="E113" s="2" t="n"/>
+    </row>
+    <row r="114">
+      <c r="E114" s="2" t="n"/>
+    </row>
+    <row r="115">
+      <c r="E115" s="2" t="n"/>
+    </row>
+    <row r="116">
+      <c r="E116" s="2" t="n"/>
+    </row>
+    <row r="117">
+      <c r="E117" s="2" t="n"/>
+    </row>
+    <row r="118">
+      <c r="E118" s="2" t="n"/>
+    </row>
+    <row r="119">
+      <c r="E119" s="2" t="n"/>
+    </row>
+    <row r="120">
+      <c r="E120" s="2" t="n"/>
+    </row>
+    <row r="121">
+      <c r="E121" s="2" t="n"/>
+    </row>
+    <row r="122">
+      <c r="E122" s="2" t="n"/>
+    </row>
+    <row r="123">
+      <c r="E123" s="2" t="n"/>
+    </row>
+    <row r="124">
+      <c r="E124" s="2" t="n"/>
+    </row>
+    <row r="125">
+      <c r="E125" s="2" t="n"/>
+    </row>
+    <row r="126">
+      <c r="E126" s="2" t="n"/>
+    </row>
+    <row r="127">
+      <c r="E127" s="2" t="n"/>
+    </row>
+    <row r="128">
+      <c r="E128" s="2" t="n"/>
+    </row>
+    <row r="129">
+      <c r="E129" s="2" t="n"/>
+    </row>
+    <row r="130">
+      <c r="E130" s="2" t="n"/>
+    </row>
+    <row r="131">
+      <c r="E131" s="2" t="n"/>
+    </row>
+    <row r="132">
+      <c r="E132" s="2" t="n"/>
+    </row>
+    <row r="133">
+      <c r="E133" s="2" t="n"/>
+    </row>
+    <row r="134">
+      <c r="E134" s="2" t="n"/>
+    </row>
+    <row r="135">
+      <c r="E135" s="2" t="n"/>
+    </row>
+    <row r="136">
+      <c r="E136" s="2" t="n"/>
+    </row>
+    <row r="137">
+      <c r="E137" s="2" t="n"/>
+    </row>
+    <row r="138">
+      <c r="E138" s="2" t="n"/>
+    </row>
+    <row r="139">
+      <c r="E139" s="2" t="n"/>
+    </row>
+    <row r="140">
+      <c r="E140" s="2" t="n"/>
+    </row>
+    <row r="141">
+      <c r="E141" s="2" t="n"/>
+    </row>
+    <row r="142">
+      <c r="E142" s="2" t="n"/>
+    </row>
+    <row r="143">
+      <c r="E143" s="2" t="n"/>
+    </row>
+    <row r="144">
+      <c r="E144" s="2" t="n"/>
+    </row>
+    <row r="145">
+      <c r="E145" s="2" t="n"/>
+    </row>
+    <row r="146">
+      <c r="E146" s="2" t="n"/>
+    </row>
+    <row r="147">
+      <c r="E147" s="2" t="n"/>
+    </row>
+    <row r="148">
+      <c r="E148" s="2" t="n"/>
+    </row>
+    <row r="149">
+      <c r="E149" s="2" t="n"/>
+    </row>
+    <row r="150">
+      <c r="E150" s="2" t="n"/>
+    </row>
+    <row r="151">
+      <c r="E151" s="2" t="n"/>
+    </row>
+    <row r="152">
+      <c r="E152" s="2" t="n"/>
+    </row>
+    <row r="153">
+      <c r="E153" s="2" t="n"/>
+    </row>
+    <row r="154">
+      <c r="E154" s="2" t="n"/>
+    </row>
+    <row r="155">
+      <c r="E155" s="2" t="n"/>
+    </row>
+    <row r="156">
+      <c r="E156" s="2" t="n"/>
+    </row>
+    <row r="157">
+      <c r="E157" s="2" t="n"/>
+    </row>
+    <row r="158">
+      <c r="E158" s="2" t="n"/>
+    </row>
+    <row r="159">
+      <c r="E159" s="2" t="n"/>
+    </row>
+    <row r="160">
+      <c r="E160" s="2" t="n"/>
+    </row>
+    <row r="161">
+      <c r="E161" s="2" t="n"/>
+    </row>
+    <row r="162">
+      <c r="E162" s="2" t="n"/>
+    </row>
+    <row r="163">
+      <c r="E163" s="2" t="n"/>
+    </row>
+    <row r="164">
+      <c r="E164" s="2" t="n"/>
+    </row>
+    <row r="165">
+      <c r="E165" s="2" t="n"/>
+    </row>
+    <row r="166">
+      <c r="E166" s="2" t="n"/>
+    </row>
+    <row r="167">
+      <c r="E167" s="2" t="n"/>
+    </row>
+    <row r="168">
+      <c r="E168" s="2" t="n"/>
+    </row>
+    <row r="169">
+      <c r="E169" s="2" t="n"/>
+    </row>
+    <row r="170">
+      <c r="E170" s="2" t="n"/>
+    </row>
+    <row r="171">
+      <c r="E171" s="2" t="n"/>
+    </row>
+    <row r="172">
+      <c r="E172" s="2" t="n"/>
+    </row>
+    <row r="173">
+      <c r="E173" s="2" t="n"/>
+    </row>
+    <row r="174">
+      <c r="E174" s="2" t="n"/>
+    </row>
+    <row r="175">
+      <c r="E175" s="2" t="n"/>
+    </row>
+    <row r="176">
+      <c r="E176" s="2" t="n"/>
+    </row>
+    <row r="177">
+      <c r="E177" s="2" t="n"/>
+    </row>
+    <row r="178">
+      <c r="E178" s="2" t="n"/>
+    </row>
+    <row r="179">
+      <c r="E179" s="2" t="n"/>
+    </row>
+    <row r="180">
+      <c r="E180" s="2" t="n"/>
+    </row>
+    <row r="181">
+      <c r="E181" s="2" t="n"/>
+    </row>
+    <row r="182">
+      <c r="E182" s="2" t="n"/>
+    </row>
+    <row r="183">
+      <c r="E183" s="2" t="n"/>
+    </row>
+    <row r="184">
+      <c r="E184" s="2" t="n"/>
+    </row>
+    <row r="185">
+      <c r="E185" s="2" t="n"/>
+    </row>
+    <row r="186">
+      <c r="E186" s="2" t="n"/>
+    </row>
+    <row r="187">
+      <c r="E187" s="2" t="n"/>
+    </row>
+    <row r="188">
+      <c r="E188" s="2" t="n"/>
+    </row>
+    <row r="189">
+      <c r="E189" s="2" t="n"/>
+    </row>
+    <row r="190">
+      <c r="E190" s="2" t="n"/>
+    </row>
+    <row r="191">
+      <c r="E191" s="2" t="n"/>
+    </row>
+    <row r="192">
+      <c r="E192" s="2" t="n"/>
+    </row>
+    <row r="193">
+      <c r="E193" s="2" t="n"/>
+    </row>
+    <row r="194">
+      <c r="E194" s="2" t="n"/>
+    </row>
+    <row r="195">
+      <c r="E195" s="2" t="n"/>
+    </row>
+    <row r="196">
+      <c r="E196" s="2" t="n"/>
+    </row>
+    <row r="197">
+      <c r="E197" s="2" t="n"/>
+    </row>
+    <row r="198">
+      <c r="E198" s="2" t="n"/>
+    </row>
+    <row r="199">
+      <c r="E199" s="2" t="n"/>
+    </row>
+    <row r="200">
+      <c r="E200" s="2" t="n"/>
+    </row>
+    <row r="201">
+      <c r="E201" s="2" t="n"/>
+    </row>
+    <row r="202">
+      <c r="E202" s="2" t="n"/>
+    </row>
+    <row r="203">
+      <c r="E203" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2376,94 +3574,94 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>income_role</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>income_employee</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>income_self_employed</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>income_unemployed</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>income_annual_gross</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>income_other_source_1</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>income_other_source_2</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>income_other_source_3</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>income_total_gross</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>applicant | spouse | other_family</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>Ναι | Όχι</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>Ναι | Όχι</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>Ναι | Όχι</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>€ · 10.4.6</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="I3" s="6" t="inlineStr">
         <is>
           <t>€</t>
         </is>
@@ -2570,171 +3768,171 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Άλλη ακίνητη ιδιοκτησία (α) κατοικία — Ναι</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Άλλη ακίνητη ιδιοκτησία (α) — επεξήγηση</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Άλλη ακίνητη ιδιοκτησία (β) οικόπεδο/γη — Ναι</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Άλλη ακίνητη ιδιοκτησία (β) — επεξήγηση</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Αποξένωση τελευταία 3 έτη (γ) — Ναι</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Αποξένωση (γ) — επεξήγηση</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Προηγούμενη κρατική στεγαστική βοήθεια — Ναι</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Προηγούμενη στεγαστική βοήθεια — επεξήγηση</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Άλλη αίτηση — 1η επιλογή (κοινότητα)</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Άλλη αίτηση — 2η επιλογή</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>Άλλη αίτηση — 3η επιλογή</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>Άλλες αιτήσεις — πρόσθετες πληροφορίες</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>Ενόρκως — ημερομηνία υπογραφής αίτησης</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>Ενόρκως — Έπαρχος (κείμενο)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>property_residence_yes</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>property_residence_explanation</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>property_land_yes</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>property_land_explanation</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>property_alienation_yes</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>property_alienation_explanation</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>previous_housing_aid_yes</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>previous_housing_aid_explanation</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>other_application_pref_1</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="J2" s="4" t="inlineStr">
         <is>
           <t>other_application_pref_2</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="K2" s="4" t="inlineStr">
         <is>
           <t>other_application_pref_3</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="L2" s="4" t="inlineStr">
         <is>
           <t>other_applications_notes</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="M2" s="4" t="inlineStr">
         <is>
           <t>affidavit_signed_on</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="N2" s="4" t="inlineStr">
         <is>
           <t>affidavit_district_office</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>Ναι | Όχι · 10.4.4</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>Ναι | Όχι</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>Ναι | Όχι · 10.4.5</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>Ναι | Όχι · 10.4.7</t>
         </is>
       </c>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="M3" s="5" t="inlineStr">
         <is>
           <t>YYYY-MM-DD · αρχείο μόνο</t>
         </is>

</xml_diff>